<commit_message>
C_class tourne. Reste à équilibrer et ajouter les dictionnaire de puissance
</commit_message>
<xml_diff>
--- a/example/GRAFS_project_example_C.xlsx
+++ b/example/GRAFS_project_example_C.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FF7C76-B34F-44E0-A889-AB517AF7C79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FE3735-47F4-4A3B-91CE-D8B49F33B5DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -348,9 +348,6 @@
     <t>Bio_diet</t>
   </si>
   <si>
-    <t>CO2 share (%)</t>
-  </si>
-  <si>
     <t>Target Energy Production (GWh)</t>
   </si>
   <si>
@@ -358,6 +355,9 @@
   </si>
   <si>
     <t>Weight energy inputs</t>
+  </si>
+  <si>
+    <t>Share CO2 (%)</t>
   </si>
 </sst>
 </file>
@@ -1374,13 +1374,13 @@
         <v>96</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -2105,7 +2105,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -2113,7 +2113,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B9">
         <v>1</v>

</xml_diff>

<commit_message>
Des progrès. Mise en place des mécanismes pour le mode prospective. Il faut continuer, débug et vérifier que les colonnes de sorties collent au mode historique. Gérer les flux de en post_opti aussi.
</commit_message>
<xml_diff>
--- a/example/GRAFS_project_example_C.xlsx
+++ b/example/GRAFS_project_example_C.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94166A49-0460-455B-A965-394CF969B4E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C710D653-F824-4E2D-941F-3B9935FF9A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16530" yWindow="-15870" windowWidth="25440" windowHeight="15270" activeTab="6" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="104">
   <si>
     <t>Culture</t>
   </si>
@@ -319,9 +319,6 @@
   </si>
   <si>
     <t>Seed input (ktN/ktN)</t>
-  </si>
-  <si>
-    <t>Energy Production (MWh/tFW)</t>
   </si>
   <si>
     <t>Facility</t>
@@ -1369,33 +1366,33 @@
   <sheetData>
     <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>94</v>
-      </c>
       <c r="C1" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
         <v>95</v>
-      </c>
-      <c r="B2" t="s">
-        <v>96</v>
       </c>
       <c r="C2">
         <v>1000</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -1403,16 +1400,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
         <v>97</v>
-      </c>
-      <c r="B3" t="s">
-        <v>98</v>
       </c>
       <c r="C3">
         <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -1425,7 +1422,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58CEBB00-B56F-4BED-97E3-E735E21789EF}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28.1796875" customWidth="1"/>
@@ -1434,11 +1431,10 @@
     <col min="4" max="4" width="16.08984375" customWidth="1"/>
     <col min="6" max="6" width="13.08984375" customWidth="1"/>
     <col min="9" max="9" width="24" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
-    <col min="11" max="11" width="19.81640625" customWidth="1"/>
+    <col min="10" max="10" width="19.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>56</v>
       </c>
@@ -1467,13 +1463,10 @@
         <v>70</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="K1" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -1496,13 +1489,10 @@
         <v>46</v>
       </c>
       <c r="J2">
-        <v>0.23</v>
-      </c>
-      <c r="K2">
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -1522,13 +1512,10 @@
         <v>26</v>
       </c>
       <c r="J3">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="K3">
         <v>0.3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -1550,11 +1537,8 @@
       <c r="J4">
         <v>0</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -1574,13 +1558,10 @@
         <v>20</v>
       </c>
       <c r="J5">
-        <v>0.54</v>
-      </c>
-      <c r="K5">
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -1600,13 +1581,10 @@
         <v>10</v>
       </c>
       <c r="J6">
-        <v>0.21</v>
-      </c>
-      <c r="K6">
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -1626,9 +1604,6 @@
         <v>26</v>
       </c>
       <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
         <v>0</v>
       </c>
     </row>
@@ -1639,7 +1614,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9008F097-1A19-4A13-A439-D292DC31E615}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38.453125" customWidth="1"/>
@@ -1648,10 +1623,9 @@
     <col min="5" max="5" width="19.1796875" customWidth="1"/>
     <col min="6" max="6" width="18.1796875" customWidth="1"/>
     <col min="8" max="8" width="14.7265625" customWidth="1"/>
-    <col min="9" max="9" width="28.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>16</v>
       </c>
@@ -1677,13 +1651,10 @@
         <v>80</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="J1" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1708,11 +1679,8 @@
       <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1737,11 +1705,8 @@
       <c r="H3">
         <v>0</v>
       </c>
-      <c r="I3">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1766,11 +1731,8 @@
       <c r="H4">
         <v>0</v>
       </c>
-      <c r="I4">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1795,11 +1757,8 @@
       <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -1824,11 +1783,8 @@
       <c r="H6">
         <v>0</v>
       </c>
-      <c r="I6">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -1853,11 +1809,8 @@
       <c r="H7">
         <v>0</v>
       </c>
-      <c r="I7">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -1882,11 +1835,8 @@
       <c r="H8">
         <v>2</v>
       </c>
-      <c r="I8">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1911,11 +1861,8 @@
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
@@ -1940,11 +1887,8 @@
       <c r="H10">
         <v>0</v>
       </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -1969,11 +1913,8 @@
       <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -1998,11 +1939,8 @@
       <c r="H12">
         <v>0</v>
       </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -2028,9 +1966,6 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>0.25</v>
-      </c>
-      <c r="J13">
         <v>0</v>
       </c>
     </row>
@@ -2098,7 +2033,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -2106,7 +2041,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8">
         <v>0.1</v>
@@ -2114,7 +2049,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -2138,7 +2073,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B12">
         <v>1</v>

</xml_diff>

<commit_message>
Mise à jour de la couche carbone (suppression de roots production pour homogénéiser les calculs de résidus et de racines)
</commit_message>
<xml_diff>
--- a/example/GRAFS_project_example_C.xlsx
+++ b/example/GRAFS_project_example_C.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD117925-C191-4A52-A398-20DD9FA4B5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533B3848-71A4-4963-9EF7-D946E8363D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16530" yWindow="-15870" windowWidth="25440" windowHeight="15270" activeTab="4" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="16530" yWindow="-15870" windowWidth="25440" windowHeight="15270" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="103">
   <si>
     <t>Culture</t>
   </si>
@@ -271,9 +271,6 @@
   </si>
   <si>
     <t>Carbon Mechanisation Intensity (ktC/ha)</t>
-  </si>
-  <si>
-    <t>Surface Root Production (kgC/ha)</t>
   </si>
   <si>
     <t>Residue Humification Coefficient (%)</t>
@@ -773,7 +770,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.54296875" customWidth="1"/>
@@ -786,10 +783,9 @@
     <col min="11" max="12" width="25.54296875" customWidth="1"/>
     <col min="13" max="14" width="37.81640625" customWidth="1"/>
     <col min="15" max="15" width="32.1796875" customWidth="1"/>
-    <col min="16" max="16" width="28.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -818,28 +814,25 @@
         <v>52</v>
       </c>
       <c r="J1" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>75</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="P1" s="6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" ht="25" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -885,11 +878,8 @@
       <c r="O2" s="4">
         <v>22</v>
       </c>
-      <c r="P2" s="4">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:15" ht="25" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -935,11 +925,8 @@
       <c r="O3" s="4">
         <v>22</v>
       </c>
-      <c r="P3" s="4">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:15" ht="25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -985,11 +972,8 @@
       <c r="O4" s="4">
         <v>22</v>
       </c>
-      <c r="P4" s="4">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="25" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:15" ht="25" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1035,11 +1019,8 @@
       <c r="O5" s="4">
         <v>22</v>
       </c>
-      <c r="P5" s="4">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1085,11 +1066,8 @@
       <c r="O6" s="4">
         <v>22</v>
       </c>
-      <c r="P6" s="4">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1135,11 +1113,8 @@
       <c r="O7" s="4">
         <v>28</v>
       </c>
-      <c r="P7" s="4">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1147,7 +1122,7 @@
         <v>47</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D8" s="4">
         <v>0</v>
@@ -1185,20 +1160,17 @@
       <c r="O8" s="4">
         <v>25</v>
       </c>
-      <c r="P8" s="4">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="D9" s="1">
         <v>0</v>
       </c>
@@ -1233,9 +1205,6 @@
         <v>0</v>
       </c>
       <c r="O9" s="4">
-        <v>0</v>
-      </c>
-      <c r="P9" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1367,33 +1336,33 @@
   <sheetData>
     <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>93</v>
-      </c>
       <c r="C1" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" t="s">
         <v>94</v>
-      </c>
-      <c r="B2" t="s">
-        <v>95</v>
       </c>
       <c r="C2">
         <v>1000</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -1401,16 +1370,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" t="s">
         <v>96</v>
-      </c>
-      <c r="B3" t="s">
-        <v>97</v>
       </c>
       <c r="C3">
         <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -1646,13 +1615,13 @@
         <v>54</v>
       </c>
       <c r="G1" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="I1" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1822,7 +1791,7 @@
         <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E8">
         <v>2.0499999999999998</v>
@@ -1943,16 +1912,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" t="s">
         <v>85</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
       </c>
       <c r="C13" t="s">
         <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -2034,7 +2003,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -2042,7 +2011,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B8">
         <v>0.1</v>
@@ -2050,7 +2019,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -2058,7 +2027,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -2066,7 +2035,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -2074,7 +2043,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B12">
         <v>1</v>

</xml_diff>